<commit_message>
V112: enumerate all thirty-nine anatomy species, formulas and generated signal resources
</commit_message>
<xml_diff>
--- a/docs/YAUTJA_V112_MECANIQUES_CHASSE.xlsx
+++ b/docs/YAUTJA_V112_MECANIQUES_CHASSE.xlsx
@@ -1840,7 +1840,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultRowHeight="36"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -2250,8 +2250,136 @@
         </is>
       </c>
     </row>
+    <row r="16" ht="42" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ART112-01</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Symbole visual</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SVG original généré par scripts/build-discovery-signals-v112.mjs ; dessin vectoriel natif et libellé texte dans le Canvas.</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">public/game/assets/v112/discovery/visual.svg</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ressource d'export/reproductibilité ; le rendu en jeu ne dépend pas de la réussite d'un chargement d'image.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="42" customHeight="1">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ART112-02</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Symbole radio</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SVG original généré par scripts/build-discovery-signals-v112.mjs ; dessin vectoriel natif et libellé texte dans le Canvas.</t>
+        </is>
+      </c>
+      <c r="E17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">public/game/assets/v112/discovery/radio.svg</t>
+        </is>
+      </c>
+      <c r="F17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ressource d'export/reproductibilité ; le rendu en jeu ne dépend pas de la réussite d'un chargement d'image.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="42" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ART112-03</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Symbole scent</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SVG original généré par scripts/build-discovery-signals-v112.mjs ; dessin vectoriel natif et libellé texte dans le Canvas.</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">public/game/assets/v112/discovery/scent.svg</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ressource d'export/reproductibilité ; le rendu en jeu ne dépend pas de la réussite d'un chargement d'image.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="42" customHeight="1">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ART112-04</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Symbole animal</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SVG original généré par scripts/build-discovery-signals-v112.mjs ; dessin vectoriel natif et libellé texte dans le Canvas.</t>
+        </is>
+      </c>
+      <c r="E19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">public/game/assets/v112/discovery/animal.svg</t>
+        </is>
+      </c>
+      <c r="F19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ressource d'export/reproductibilité ; le rendu en jeu ne dépend pas de la réussite d'un chargement d'image.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:F15"/>
+  <autoFilter ref="A4:F19"/>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
@@ -2268,6 +2396,10 @@
     <hyperlink ref="E13" r:id="rId9" tooltip="Ouvrir la source GitHub"/>
     <hyperlink ref="E14" r:id="rId10" tooltip="Ouvrir la source GitHub"/>
     <hyperlink ref="E15" r:id="rId11" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E16" r:id="rId12" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E17" r:id="rId13" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E18" r:id="rId14" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E19" r:id="rId15" tooltip="Ouvrir la source GitHub"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.2" footer="0.2"/>
@@ -11451,7 +11583,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr defaultRowHeight="36"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -11957,8 +12089,1401 @@
         </is>
       </c>
     </row>
+    <row r="19" ht="42" customHeight="1">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-01</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hell-hound-stalker</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cuir de chien de chasse : 2.4 kg ; 3 volume(s) ; 3.8 s ; fragilité 1 ; dépeçage requis
+Tendon de poursuite : 0.4 kg ; 1 volume(s) ; 2.6 s ; fragilité 1.3 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="42" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-02</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cinder-12--hell-hound-stalker</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cuir de chien de chasse : 2.4 kg ; 3 volume(s) ; 3.8 s ; fragilité 1 ; dépeçage requis
+Tendon de poursuite : 0.4 kg ; 1 volume(s) ; 2.6 s ; fragilité 1.3 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="42" customHeight="1">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-03</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">razorback-grazer</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peau de brouteur : 3.8 kg ; 3 volume(s) ; 3.8 s ; fragilité 1 ; dépeçage requis
+Côte dorsale : 1.2 kg ; 2 volume(s) ; 3.4 s ; fragilité 0.55 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="42" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-04</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nivalis-k--razorback-grazer</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peau de brouteur : 3.8 kg ; 3 volume(s) ; 3.8 s ; fragilité 1 ; dépeçage requis
+Côte dorsale : 1.2 kg ; 2 volume(s) ; 3.4 s ; fragilité 0.55 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="42" customHeight="1">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-05</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">oseris-iv--vineback-grazer</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peau à fibres végétales : 3.2 kg ; 3 volume(s) ; 3.8 s ; fragilité 1 ; dépeçage requis
+Ligament dorsal : 0.4 kg ; 1 volume(s) ; 2.6 s ; fragilité 1.3 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E23" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F23" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="42" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-06</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">oseris-iv--mist-pouncer</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pelage de bondisseur : 2.4 kg ; 3 volume(s) ; 3.8 s ; fragilité 1 ; dépeçage requis
+Tendon de bond : 0.4 kg ; 1 volume(s) ; 2.6 s ; fragilité 1.3 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="42" customHeight="1">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-07</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">oseris-iv--mirror-chameleon</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peau chromatophore : 1.6 kg ; 3 volume(s) ; 3.8 s ; fragilité 1 ; dépeçage requis
+Échantillon pigmentaire : 0.4 kg ; 1 volume(s) ; 2.6 s ; fragilité 1.3 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E25" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F25" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="42" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-08</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">naraka-delta--reed-cat</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pelage palustre : 1.8 kg ; 3 volume(s) ; 3.8 s ; fragilité 1 ; dépeçage requis
+Tendon félin : 0.4 kg ; 1 volume(s) ; 2.6 s ; fragilité 1.3 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="42" customHeight="1">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-09</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">serekh-9--dust-jackal</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pelage filtrant : 1.8 kg ; 3 volume(s) ; 3.8 s ; fragilité 1 ; dépeçage requis
+Os nasal secondaire : 1.2 kg ; 2 volume(s) ; 3.4 s ; fragilité 0.55 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E27" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F27" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="42" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-10</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nivalis-k--snow-prowler</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fourrure isolante : 2.8 kg ; 3 volume(s) ; 3.8 s ; fragilité 1 ; dépeçage requis
+Tissu thermorégulateur : 0.4 kg ; 1 volume(s) ; 2.6 s ; fragilité 1.3 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="42" customHeight="1">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-11</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nivalis-k--glacier-ram</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cuir de bélier : 4 kg ; 3 volume(s) ; 3.8 s ; fragilité 1 ; dépeçage requis
+Côte renforcée : 1.2 kg ; 2 volume(s) ; 3.4 s ; fragilité 0.55 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E29" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F29" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="42" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-12</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cinder-12--basalt-ram</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cuir de bélier : 4 kg ; 3 volume(s) ; 3.8 s ; fragilité 1 ; dépeçage requis
+Côte renforcée : 1.2 kg ; 2 volume(s) ; 3.4 s ; fragilité 0.55 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="42" customHeight="1">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-13</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">serekh-9--salt-ram</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cuir de bélier : 4 kg ; 3 volume(s) ; 3.8 s ; fragilité 1 ; dépeçage requis
+Côte renforcée : 1.2 kg ; 2 volume(s) ; 3.4 s ; fragilité 0.55 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E31" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F31" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="42" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-14</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">xeno-drone</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Segment caudal de xénomorphe : 1.2 kg ; 2 volume(s) ; 3.4 s ; fragilité 0.55 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="42" customHeight="1">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-15</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">common--wandering-xeno-drone</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Segment caudal de xénomorphe : 1.2 kg ; 2 volume(s) ; 3.4 s ; fragilité 0.55 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E33" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F33" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="42" customHeight="1">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-16</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">oseris-iv--jungle-xeno-scout</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Segment caudal de xénomorphe : 1.2 kg ; 2 volume(s) ; 3.4 s ; fragilité 0.55 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="42" customHeight="1">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-17</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nivalis-k--frost-xeno</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Segment caudal de xénomorphe : 1.2 kg ; 2 volume(s) ; 3.4 s ; fragilité 0.55 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E35" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F35" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="42" customHeight="1">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-18</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cinder-12--scorch-xeno</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Segment caudal de xénomorphe : 1.2 kg ; 2 volume(s) ; 3.4 s ; fragilité 0.55 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="42" customHeight="1">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-19</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">acheron-sigma--temple-xeno</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Segment caudal de xénomorphe : 1.2 kg ; 2 volume(s) ; 3.4 s ; fragilité 0.55 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E37" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F37" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="42" customHeight="1">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-20</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pelagos-m--swimmer-xeno</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Segment caudal de xénomorphe : 1.2 kg ; 2 volume(s) ; 3.4 s ; fragilité 0.55 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="42" customHeight="1">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-21</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">xeno-praetorian</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Éperon thoracique : 1.2 kg ; 2 volume(s) ; 3.4 s ; fragilité 0.55 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E39" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F39" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="42" customHeight="1">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-22</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">oseris-iv--needle-frog</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tissu glandulaire d'aiguillon : 0.4 kg ; 1 volume(s) ; 2.6 s ; fragilité 1.3 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="42" customHeight="1">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-23</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">naraka-delta--lantern-toad</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tissu photophore : 0.4 kg ; 1 volume(s) ; 2.6 s ; fragilité 1.3 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E41" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F41" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="42" customHeight="1">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-24</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pelagos-m--storm-eel</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tissu électrocyte : 0.4 kg ; 1 volume(s) ; 2.6 s ; fragilité 1.3 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="42" customHeight="1">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-25</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">naraka-delta--sludge-eel</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tissu électrocyte : 0.4 kg ; 1 volume(s) ; 2.6 s ; fragilité 1.3 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E43" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F43" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="42" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-26</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bonecrest-ravager</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cuir du ravageur : 4.2 kg ; 3 volume(s) ; 3.8 s ; fragilité 1 ; dépeçage requis
+Phalange de soutien : 1.2 kg ; 2 volume(s) ; 3.4 s ; fragilité 0.55 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="42" customHeight="1">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-27</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">amber-mire-lurker</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peau du guetteur palustre : 3.6 kg ; 3 volume(s) ; 3.8 s ; fragilité 1 ; dépeçage requis</t>
+        </is>
+      </c>
+      <c r="E45" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F45" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="42" customHeight="1">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-28</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">naraka-delta--bog-stalker</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peau du guetteur palustre : 3.6 kg ; 3 volume(s) ; 3.8 s ; fragilité 1 ; dépeçage requis</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="42" customHeight="1">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-29</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">naraka-delta--iron-croc</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cuir à plaques ferriques : 4.4 kg ; 3 volume(s) ; 3.8 s ; fragilité 1 ; dépeçage requis
+Vertèbre terminale : 1.2 kg ; 2 volume(s) ; 3.4 s ; fragilité 0.55 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E47" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F47" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="42" customHeight="1">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-30</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">naraka-delta--fen-leaper</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peau du sauteur : 1.5 kg ; 3 volume(s) ; 3.8 s ; fragilité 1 ; dépeçage requis</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="42" customHeight="1">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-31</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">serekh-9--quill-lizard</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peau du lézard : 1.4 kg ; 3 volume(s) ; 3.8 s ; fragilité 1 ; dépeçage requis</t>
+        </is>
+      </c>
+      <c r="E49" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F49" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="42" customHeight="1">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-32</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">serekh-9--dune-strider</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tendon d'échassier : 0.4 kg ; 1 volume(s) ; 2.6 s ; fragilité 1.3 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="42" customHeight="1">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-33</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cinder-12--smoke-wyvern</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Membrane de vol : 3.8 kg ; 3 volume(s) ; 3.8 s ; fragilité 1 ; dépeçage requis</t>
+        </is>
+      </c>
+      <c r="E51" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F51" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="42" customHeight="1">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-34</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pelagos-m--razor-shark</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peau denticulée : 3 kg ; 3 volume(s) ; 3.8 s ; fragilité 1 ; dépeçage requis
+Tissu sensoriel : 0.4 kg ; 1 volume(s) ; 2.6 s ; fragilité 1.3 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="42" customHeight="1">
+      <c r="A53" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-35</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C53" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">oseris-iv--thunder-macaque</t>
+        </is>
+      </c>
+      <c r="D53" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pelage du dominant : 2.6 kg ; 3 volume(s) ; 3.8 s ; fragilité 1 ; dépeçage requis
+Phalange du dominant : 1.2 kg ; 2 volume(s) ; 3.4 s ; fragilité 0.55 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E53" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F53" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="42" customHeight="1">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-36</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mycora-v--spore-hound</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Culture mycélienne canine : 0.4 kg ; 1 volume(s) ; 2.6 s ; fragilité 1.3 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="42" customHeight="1">
+      <c r="A55" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-37</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C55" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mycora-v--glow-moth</t>
+        </is>
+      </c>
+      <c r="D55" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Poudre phosphorescente : 0.4 kg ; 1 volume(s) ; 2.6 s ; fragilité 1.3 ; dépeçage non requis</t>
+        </is>
+      </c>
+      <c r="E55" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F55" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="42" customHeight="1">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-38</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pelagos-m--hunter-manta</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Membrane alaire : 1.2 kg ; 3 volume(s) ; 3.8 s ; fragilité 1 ; dépeçage requis</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="42" customHeight="1">
+      <c r="A57" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-39</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C57" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nivalis-k--frost-manta</t>
+        </is>
+      </c>
+      <c r="D57" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Membrane alaire : 1.2 kg ; 3 volume(s) ; 3.8 s ; fragilité 1 ; dépeçage requis</t>
+        </is>
+      </c>
+      <c r="E57" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F57" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock d'une pièce par partie et par corps réel ; la reprise et l'extraction conservent la même identité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="42" customHeight="1">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ANA112-15</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Perte d'intégrité : formule</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Perte cumulée = clamp(perte + dégâts/santéMax × (9 mêlée ou 28 arme) + surkill/santéMax ×45, 0, 100). Intégrité = arrondi(100-perte).</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Les nombres sont des réglages du fan game ; tous les coups réels contribuent, pas seulement le dernier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="42" customHeight="1">
+      <c r="A59" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ANA112-16</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C59" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qualité de pièce : formule</t>
+        </is>
+      </c>
+      <c r="D59" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qualité = arrondi(clamp(100-(100-intégrité)×fragilité-(analyse absente ?12:0),0,100)).</t>
+        </is>
+      </c>
+      <c r="E59" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F59" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Même dégâts, partie et analyse produisent la même qualité ; aucun aléa à la reprise.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="42" customHeight="1">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ANA112-17</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Masse corporelle : formule</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Masse = arrondi(clamp(largeur×hauteur/60,12,300)) kg. Humain66×94≈103 kg ; Yautja74×112≈138 kg ; chien104×84≈146 kg.</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adaptation de gameplay dimensionnelle ; pas une estimation canonique de masse réelle. Portage maximal170 kg.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="42" customHeight="1">
+      <c r="A61" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT112-00</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C61" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espèce absente du catalogue</t>
+        </is>
+      </c>
+      <c r="D61" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aucune partie anatomique supplémentaire pour une espèce non listée, notamment humain, synthétique ou végétal absent de la table.</t>
+        </is>
+      </c>
+      <c r="E61" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">app/game/systems/anatomyHarvestV112.ts</t>
+        </is>
+      </c>
+      <c r="F61" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La définition d'un trophée historique reste indépendante ; aucun tissu ou peau universels.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:F18"/>
+  <autoFilter ref="A4:F61"/>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
@@ -11978,6 +13503,49 @@
     <hyperlink ref="E16" r:id="rId12" tooltip="Ouvrir la source GitHub"/>
     <hyperlink ref="E17" r:id="rId13" tooltip="Ouvrir la source GitHub"/>
     <hyperlink ref="E18" r:id="rId14" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E19" r:id="rId15" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E20" r:id="rId16" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E21" r:id="rId17" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E22" r:id="rId18" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E23" r:id="rId19" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E24" r:id="rId20" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E25" r:id="rId21" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E26" r:id="rId22" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E27" r:id="rId23" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E28" r:id="rId24" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E29" r:id="rId25" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E30" r:id="rId26" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E31" r:id="rId27" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E32" r:id="rId28" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E33" r:id="rId29" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E34" r:id="rId30" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E35" r:id="rId31" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E36" r:id="rId32" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E37" r:id="rId33" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E38" r:id="rId34" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E39" r:id="rId35" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E40" r:id="rId36" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E41" r:id="rId37" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E42" r:id="rId38" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E43" r:id="rId39" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E44" r:id="rId40" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E45" r:id="rId41" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E46" r:id="rId42" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E47" r:id="rId43" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E48" r:id="rId44" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E49" r:id="rId45" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E50" r:id="rId46" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E51" r:id="rId47" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E52" r:id="rId48" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E53" r:id="rId49" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E54" r:id="rId50" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E55" r:id="rId51" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E56" r:id="rId52" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E57" r:id="rId53" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E58" r:id="rId54" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E59" r:id="rId55" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E60" r:id="rId56" tooltip="Ouvrir la source GitHub"/>
+    <hyperlink ref="E61" r:id="rId57" tooltip="Ouvrir la source GitHub"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.2" footer="0.2"/>

</xml_diff>

<commit_message>
docs(V112): preserve executed hunting evidence, five captures and exhaustive workbook
</commit_message>
<xml_diff>
--- a/docs/YAUTJA_V112_MECANIQUES_CHASSE.xlsx
+++ b/docs/YAUTJA_V112_MECANIQUES_CHASSE.xlsx
@@ -297,7 +297,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Commit96 ba117 a35 b54142640 ad2915 fe3 e9847 fe060 ad.</t>
+          <t xml:space="preserve">Commit de base 96ba117a35b54142640ad2915fe3e9847fe060ad, PR21 fusionnée.</t>
         </is>
       </c>
     </row>
@@ -531,9 +531,9 @@
           <t xml:space="preserve">SRC112-10</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NON_QUALIFIE</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -676,7 +676,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="36" customHeight="1">
+    <row r="6" ht="42" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">OUT112-02</t>
@@ -694,7 +694,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Coût appliqué au succès confirmé seulement.</t>
+          <t xml:space="preserve">Usure de 5 points par dépeçage ou prélèvement anatomique achevé, y compris si la mission échoue ou est abandonnée ensuite.</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -704,7 +704,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Démarrer ou interrompre ne paie pas le succès.</t>
+          <t xml:space="preserve">Démarrer ou interrompre use de 0 point ; analyse, marque, suspension et gestes d'atelier ne sont pas ce coût.</t>
         </is>
       </c>
     </row>
@@ -800,7 +800,7 @@
       </c>
       <c r="F9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Débit et état confirmés ensemble avant succès.</t>
+          <t xml:space="preserve">Coût nul, même à zéro marque ; condition remise à 100 après confirmation de l'enregistrement.</t>
         </is>
       </c>
     </row>
@@ -836,7 +836,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="36" customHeight="1">
+    <row r="11" ht="42" customHeight="1">
       <c r="A11" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">OUT112-07</t>
@@ -854,7 +854,7 @@
       </c>
       <c r="D11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Solde insuffisant ou opération répétée ne mute pas la sauvegarde.</t>
+          <t xml:space="preserve">Une écriture refusée ne confirme pas l'affûtage ; les réducteurs normalisent l'état courant.</t>
         </is>
       </c>
       <c r="E11" s="0" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="F11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Double clic utilise le dernier état confirmé.</t>
+          <t xml:space="preserve">Double clic utilise le dernier état confirmé et ne crée ni marque ni pièce.</t>
         </is>
       </c>
     </row>
@@ -1681,7 +1681,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="36" customHeight="1">
+    <row r="13" ht="57" customHeight="1">
       <c r="A13" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">ACC112-09</t>
@@ -1699,7 +1699,7 @@
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Affectation manette avec permutation anti-conflit.</t>
+          <t xml:space="preserve">Douze affectations manette permutées sans conflit ; Bas+Interagir ouvre le menu d'un corps voisin.</t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr">
@@ -1709,7 +1709,7 @@
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ancien bouton ne continue pas d'agir silencieusement.</t>
+          <t xml:space="preserve">Navigation Haut/Bas, Saut affecté confirme, Interagir affecté ferme ; les événements du pad sont consommés sans effacer les commandes clavier/tactiles concurrentes.</t>
         </is>
       </c>
     </row>
@@ -1745,7 +1745,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="36" customHeight="1">
+    <row r="15" ht="42" customHeight="1">
       <c r="A15" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">ACC112-11</t>
@@ -1763,49 +1763,49 @@
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Réglages et sortie atteignables à390 px.</t>
+          <t xml:space="preserve">Réglages et sortie atteignables dans le viewport Chromium de 390 px.</t>
         </is>
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">app/game/HuntAccessibilityPanelV112.tsx</t>
+        </is>
+      </c>
+      <c r="F15" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pas de débordement horizontal ; défilement normal. Aucun téléphone physique qualifié.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="42" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ACC112-12</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Score</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Les effets des options sur score sont explicités.</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">app/game/systems/huntAccessibilityV112.ts</t>
         </is>
       </c>
-      <c r="F15" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pas de contrôle indispensable hors écran.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="36" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ACC112-12</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Score</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Les effets des options sur score sont explicités.</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">app/game/systems/huntAccessibilityV112.ts</t>
-        </is>
-      </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aucun malus caché lié à l'accessibilité.</t>
+          <t xml:space="preserve">Aucun coefficient de score direct ajouté par le profil ; la chasse continue et son temps peut toujours affecter le score et la qualité Apex.</t>
         </is>
       </c>
     </row>
@@ -3731,7 +3731,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="36" customHeight="1">
+    <row r="30" ht="42" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">PAR112-02</t>
@@ -3744,7 +3744,7 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Longueur minimale</t>
+          <t xml:space="preserve">Longueur admissible</t>
         </is>
       </c>
       <c r="D30" s="4">
@@ -3752,7 +3752,7 @@
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">px</t>
+          <t xml:space="preserve">px minimum ; plafond2048</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
@@ -3762,7 +3762,7 @@
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maximale bornée par la hauteur du vrai support.</t>
+          <t xml:space="preserve">Longueur maximale = min(hauteur réelle du support, 2048 px), même domaine pour attache, pas physique et snapshot.</t>
         </is>
       </c>
     </row>
@@ -6361,1297 +6361,1297 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="36" customHeight="1">
+    <row r="5" ht="87" customHeight="1">
       <c r="A5" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">QA112-01</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Outil</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ancien save sans fieldToolIds</t>
+        </is>
+      </c>
+      <c r="E5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/field-tools-rites-v111.test.mjs</t>
+        </is>
+      </c>
+      <c r="F5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/field-tools-rites-v111.test.mjs tests/field-tool-purchase-ui-v111.test.mjs tests/trophy-harvest-v111.test.mjs tests/hunt-harvest-runtime-v111.test.mjs ; Aucun outil gratuit et aucun prélèvement autorisé sans achat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="87" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-02</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Outil</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Achat à119 puis120 marques et double appel</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/field-tool-purchase-ui-v111.test.mjs</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/field-tools-rites-v111.test.mjs tests/field-tool-purchase-ui-v111.test.mjs tests/trophy-harvest-v111.test.mjs tests/hunt-harvest-runtime-v111.test.mjs ; Débit unique à120, propriété permanente et persistence confirmée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="87" customHeight="1">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-03</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dépeçage</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Préparer corps natif puis interruption</t>
+        </is>
+      </c>
+      <c r="E7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/hunt-harvest-runtime-v111.test.mjs</t>
+        </is>
+      </c>
+      <c r="F7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/field-tools-rites-v111.test.mjs tests/field-tool-purchase-ui-v111.test.mjs tests/trophy-harvest-v111.test.mjs tests/hunt-harvest-runtime-v111.test.mjs ; Geste3,2 s ajusté usure, annulation sans succès ni coût d'opération achevée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="87" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-04</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trophées</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proie haute, morte puis tombante</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/hunt-harvest-runtime-v111.test.mjs</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/field-tools-rites-v111.test.mjs tests/field-tool-purchase-ui-v111.test.mjs tests/trophy-harvest-v111.test.mjs tests/hunt-harvest-runtime-v111.test.mjs ; Prélèvement suit source réelle et ne traverse pas de mur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="72" customHeight="1">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-05</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pendule</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entrée clavier normalisée : accroche, pompage, lâcher</t>
+        </is>
+      </c>
+      <c r="E9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/hunt-canopy-runtime-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; Simulation native, vitesse tangentielle et verrou anti-réaccroche ; les adaptateurs d'entrée ne qualifient pas un clavier physique.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="72" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-06</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pendule</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entrée tactile normalisée : accroche, pompage, lâcher</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/hunt-canopy-runtime-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; Même simulation native et coûts ; injection InputHub et pointeur de fixture, sans téléphone physique.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="72" customHeight="1">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-07</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pendule</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entrée manette normalisée : accroche, pompage, lâcher</t>
+        </is>
+      </c>
+      <c r="E11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/hunt-canopy-runtime-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; Simulation native ; polling réel testé séparément au navigateur avec manette émulée, sans contrôleur physique.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="57" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-08</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pendule</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pompage borné et friction sans entrée</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/canopy-traversal-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; Vitesse plafonnée ; sans entrée pas de gain d'énergie.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="87" customHeight="1">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-09</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pendule</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paroi, support absent, grand delta et longues lianes Oseris</t>
+        </is>
+      </c>
+      <c r="E13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/canopy-traversal-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; Tests purs sur vrais supports862/1054 px et frontière2048 ; attache, reeling et validateur partagent le même domaine, refus gracieux au-delà et sur données invalides. Pas de traversée ni état non fini.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="87" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-10</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pendule</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Checkpoint pendant balancement</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/hunt-canopy-runtime-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; Checkpoint réel et reprise sur Oseris déverrouillé aux longueurs760/900 px : 19 pas, puis lâcher sans boost. Longueur&gt;2048, angle/ancrage invalides refusés, aucune impulsion rejouée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="72" customHeight="1">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-11</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pendule</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Épuisement et Haut maintenu</t>
+        </is>
+      </c>
+      <c r="E15" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/hunt-canopy-runtime-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F15" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; Chute puis vraie réception requise ; pas de réaccroche aérienne.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="102" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-12</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Route</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8 missions ×3 armures ×3 sources d'entrée</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/hunt-canopy-runtime-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; 72 traversées natives isolées : ennemis retirés, état placé au pied de l'entrée, puis sol→grimpée→six contacts réels→sol sans repositionnement ; trois armures et trois InputHub normalisés. Aucune chasse complète revendiquée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="72" customHeight="1">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-13</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Route</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Routes dans world final après exploration</t>
+        </is>
+      </c>
+      <c r="E17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/canopy-traversal-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; Au moins une séquence réelle de six repos par mission ; repli terrain conservé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="72" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-14</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Carcasse</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mort réelle-&gt;analyse-&gt;flay-&gt;carry-&gt;hang</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/hunt-carcass-runtime-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; Un acteur et un corps, ancrage socket puis chute si support supprimé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="57" customHeight="1">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-15</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Carcasse</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Masse/surface/socket invalide</t>
+        </is>
+      </c>
+      <c r="E19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/carcass-anatomy-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; Refus sans déplacer ni dupliquer la carcasse.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="57" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-16</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Carcasse</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transport vers espace bloqué</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/hunt-carcass-runtime-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; Relâche le même corps sans traverser le mur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="87" customHeight="1">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-17</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Carcasse</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Suspension checkpoint source absente</t>
+        </is>
+      </c>
+      <c r="E21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/hunt-carcass-runtime-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; Mort réelle→préparation→portage→suspension→checkpoint ; restore de production admet les acteurs puis refuse le même registre si seul l'acteur source est retiré, sans mutation entrante.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="72" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-18</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Anatomie</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Catalogue espèces et parties compatibles</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/carcass-anatomy-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; Stock explicite ; synthétique sans chair et xéno sans peau universelle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="72" customHeight="1">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-19</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Anatomie</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dommages mêlée/tir/surkill et analyse</t>
+        </is>
+      </c>
+      <c r="E23" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/carcass-anatomy-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F23" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; Qualité reproductible annoncée, pas de nouveau tirage sur reload.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="57" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-20</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Anatomie</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interruption/dépôt plein avant dernier tick</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/hunt-carcass-runtime-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; Aucune partie consommée ni prise inventée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="72" customHeight="1">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-21</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Anatomie</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prélèvement puis succès/échec</t>
+        </is>
+      </c>
+      <c r="E25" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/hunt-carcass-runtime-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F25" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; Succès verse identité/qualité exacte ; échec n'accorde pas le stock.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="72" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-22</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Charge</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Budgets scout24/18, hunter36/24, berserker52/30</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/harvest-inventory-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; Masses/volumes calculés depuis les pièces ; refus atomique si dépassement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="72" customHeight="1">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-23</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Charge</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Plein déplacement/saut/grimpe/bruit</t>
+        </is>
+      </c>
+      <c r="E27" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/hunt-field-load-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F27" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; Vrais updatePlayer/applyPlayerJump et HUD : plein ×.68/.84/1.6/1.8, charge recomptée ; un corps déposé avant saut cesse de peser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="87" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-24</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Charge</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dépôt/reprise physique des nouvelles parties anatomiques</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/hunt-field-stash-runtime-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; Tests purs field-stash et runtime natif : appui réel, portée/LOS/capacité, chute balayée, registre unique, reprise checkpoint dans monde recomposé, export des seuls portés. Aucun TrophyClaim obligatoire déposé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="87" customHeight="1">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-25</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entretien</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Geste de terrain achevé, interruption et reçu rejoué</t>
+        </is>
+      </c>
+      <c r="E29" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/harvest-inventory-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F29" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; Usure de 5 points par dépeçage ou prélèvement anatomique achevé, même si la mission échoue ensuite ; 0 pour geste interrompu, reçu unique et condition bornée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="72" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-26</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entretien</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Réparation outil0 et aucune marque</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/harvest-inventory-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; Avec outil à 0 et solde 0, affûtage gratuit réussi et campagne conservée ; aucune dépense de marque.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="87" customHeight="1">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-27</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Atelier</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quatre phases : coûts 2/4/3/5, gestes 3/4/5/3</t>
+        </is>
+      </c>
+      <c r="E31" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/harvest-inventory-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F31" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; Transitions manuelles ordonnées et qualité conservée ; JSON→normalizeSave→parseSaveImport sous Date simulée en 2036 ne fait progresser ni travail ni coût/temps ; seul un nouveau geste ajoute une unité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="57" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-28</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Atelier</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Double clic et erreur durabilité</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/conservation-persistence-ui-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; Coût/statut confirmés ensemble ; aucune réussite prématurée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="57" customHeight="1">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-29</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Atelier</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Archive explicite pièce montée</t>
+        </is>
+      </c>
+      <c r="E33" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/harvest-inventory-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F33" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; Réserve compte possession/qualité et libère le dépôt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="102" customHeight="1">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-30</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accessibilité</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fenêtres normal/generous/unlimited</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/hunt-accessibility-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; Fenêtres et compteurs réels ; resultFor compare neuf profils sur faits synthétiques identiques : aucun coefficient direct caché. Le score temporel diminue pareil à 2× et 4× parTime ; aucune chasse complète jouée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="72" customHeight="1">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-31</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accessibilité</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmpress/hold/toggle et annulation</t>
+        </is>
+      </c>
+      <c r="E35" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/hunt-accessibility-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F35" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; Un acte par glyph, maintien min.35 s, bascule réarmée par nouveau glyph.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="57" customHeight="1">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-32</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accessibilité</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Remapmanette +focus perdu</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/hunt-accessibility-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; Permutation sans commande perdue ; bascule désarmée au blur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="72" customHeight="1">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-33</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accessibilité</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Migration et sérialisation réglages</t>
+        </is>
+      </c>
+      <c r="E37" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/hunt-accessibility-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F37" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; Valeurs futures/malformed normalisées, latches transitoires non persistés.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="57" customHeight="1">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-34</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Écosystème</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Témoin visible vs derrière mur</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/corpse-discovery-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; Vision réelle déclenche un événement local unique.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="57" customHeight="1">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-35</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Écosystème</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Radio bornée, investigation et animaux</t>
+        </is>
+      </c>
+      <c r="E39" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/corpse-discovery-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F39" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; Profils distincts, pas de boucle oualerte globale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="57" customHeight="1">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-36</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Écosystème</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Budget et checkpoint</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/corpse-discovery-v112.test.mjs</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; File/traitement bornés et identités restaurées sans rejouer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="72" customHeight="1">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-37</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Navigateur</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paramètres natifs dans un viewport Chromium de 390 px</t>
+        </is>
+      </c>
+      <c r="E41" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/qa-hunt-mechanics-browser-v112.mjs</t>
+        </is>
+      </c>
+      <c r="F41" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit ab47a9c2d2bf4b0a866c109efa2c96f68d526de8 ; commande node scripts/qa-hunt-mechanics-browser-v112.mjs ; Contrôles React natifs, remappage et guide lisibles ; stockage localStorage du parent de fixture et capture inspectée, sans téléphone physique.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="87" customHeight="1">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-38</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Navigateur</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panneau d'atelier manuel jusqu'au montage et à la réserve</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/qa-hunt-mechanics-browser-v112.mjs</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit ab47a9c2d2bf4b0a866c109efa2c96f68d526de8 ; commande node scripts/qa-hunt-mechanics-browser-v112.mjs ; Vrai composant et réducteurs de production, parent localStorage de fixture ; écriture refusée laisse stock/progression inchangés. Durabilité GameClient vérifiée séparément par les tests AST, sans parcours complet GameClient au navigateur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="87" customHeight="1">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-39</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Navigateur</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rites natifs et menu manette par défaut puis remappée</t>
+        </is>
+      </c>
+      <c r="E43" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/qa-hunt-mechanics-browser-v112.mjs</t>
+        </is>
+      </c>
+      <c r="F43" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit ab47a9c2d2bf4b0a866c109efa2c96f68d526de8 ; commande node scripts/qa-hunt-mechanics-browser-v112.mjs ; Mort et handler AST réels ; flay interrompu/terminé. Polling→stepGame→DOM réels : Bas+Interagir ouvre, navigation et Saut activent, Interagir ferme ; simulation continue et maintien ne fuit pas vers une autre action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="87" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-40</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Navigateur</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pendule : adaptateurs clavier/pointeur et manette émulée</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/qa-hunt-mechanics-browser-v112.mjs</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit ab47a9c2d2bf4b0a866c109efa2c96f68d526de8 ; commande node scripts/qa-hunt-mechanics-browser-v112.mjs ; Clavier/pointeur de fixture alimentent les vrais bindings et mouvements ; manette utilise pollGamepad réel. Rendu de repli et vitesse de lâcher inspectés, sans cycle d'entrée complet du composant HuntCanvas ni matériel réel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="102" customHeight="1">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA112-41</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">A_EXECUTER</t>
         </is>
       </c>
-      <c r="C5" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Outil</t>
-        </is>
-      </c>
-      <c r="D5" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ancien save sans fieldToolIds</t>
-        </is>
-      </c>
-      <c r="E5" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/field-tools-rites-v111.test.mjs</t>
-        </is>
-      </c>
-      <c r="F5" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Aucun outil gratuit et aucun prélèvement autorisé sans achat.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-02</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Outil</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Achat à119 puis120 marques et double appel</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/field-tool-purchase-ui-v111.test.mjs</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Débit unique à120, propriété permanente et persistence confirmée.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-03</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C7" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Dépeçage</t>
-        </is>
-      </c>
-      <c r="D7" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Préparer corps natif puis interruption</t>
-        </is>
-      </c>
-      <c r="E7" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/hunt-harvest-runtime-v111.test.mjs</t>
-        </is>
-      </c>
-      <c r="F7" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Geste3,2 s ajusté usure, annulation sans succès ni coût d'opération achevée.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-04</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Trophées</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Proie haute, morte puis tombante</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/hunt-harvest-runtime-v111.test.mjs</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Prélèvement suit source réelle et ne traverse pas de mur.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-05</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C9" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pendule</t>
-        </is>
-      </c>
-      <c r="D9" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Clavier normalisé : accroche, pompage, lâcher</t>
-        </is>
-      </c>
-      <c r="E9" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/hunt-canopy-runtime-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F9" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vitesse tangentielle réelle, delai anti-réaccroche sans boost.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="36" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-06</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pendule</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tactile normalisé : accroche, pompage, lâcher</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/hunt-canopy-runtime-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Même simulation et coût que clavier.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="36" customHeight="1">
-      <c r="A11" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-07</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C11" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pendule</t>
-        </is>
-      </c>
-      <c r="D11" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Manette normalisée : accroche, pompage, lâcher</t>
-        </is>
-      </c>
-      <c r="E11" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/hunt-canopy-runtime-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F11" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Même simulation et coût que clavier.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="36" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-08</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pendule</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pompage borné et friction sans entrée</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/canopy-traversal-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vitesse plafonnée ; sans entrée pas de gain d'énergie.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="36" customHeight="1">
-      <c r="A13" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-09</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C13" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pendule</t>
-        </is>
-      </c>
-      <c r="D13" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Paroi, support absent et delta long</t>
-        </is>
-      </c>
-      <c r="E13" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/canopy-traversal-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F13" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pas de traversée, attache distante ni état non fini.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="36" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-10</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pendule</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Checkpoint pendant balancement</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/hunt-canopy-runtime-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reprise sans impulse gratuite ; longueur/angle/ancrage invalides refusés.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="36" customHeight="1">
-      <c r="A15" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-11</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C15" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pendule</t>
-        </is>
-      </c>
-      <c r="D15" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Épuisement et Haut maintenu</t>
-        </is>
-      </c>
-      <c r="E15" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/hunt-canopy-runtime-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F15" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chute puis vraie réception requise ; pas de réaccroche aérienne.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="42" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-12</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Route</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8 missions ×3 armures ×3 sources d'entrée</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/hunt-canopy-runtime-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sol-&gt;prise entrée-&gt;six contacts de repos-&gt;descente, sans reposition intermédiaire.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="42" customHeight="1">
-      <c r="A17" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-13</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C17" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Route</t>
-        </is>
-      </c>
-      <c r="D17" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Routes dans world final après exploration</t>
-        </is>
-      </c>
-      <c r="E17" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/canopy-traversal-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F17" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Au moins une séquence réelle de six repos par mission ; repli terrain conservé.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="36" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-14</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Carcasse</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Mort réelle-&gt;analyse-&gt;flay-&gt;carry-&gt;hang</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/hunt-carcass-runtime-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Un acteur et un corps, ancrage socket puis chute si support supprimé.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="36" customHeight="1">
-      <c r="A19" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-15</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C19" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Carcasse</t>
-        </is>
-      </c>
-      <c r="D19" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Masse/surface/socket invalide</t>
-        </is>
-      </c>
-      <c r="E19" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/carcass-anatomy-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F19" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Refus sans déplacer ni dupliquer la carcasse.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="36" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-16</t>
-        </is>
-      </c>
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Carcasse</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Transport vers espace bloqué</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/hunt-carcass-runtime-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Relâche le même corps sans traverser le mur.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="36" customHeight="1">
-      <c r="A21" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-17</t>
-        </is>
-      </c>
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C21" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Carcasse</t>
-        </is>
-      </c>
-      <c r="D21" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Suspension checkpoint source absente</t>
-        </is>
-      </c>
-      <c r="E21" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/carcass-anatomy-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F21" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Restore revalide support, capacité, acteur et position.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="36" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-18</t>
-        </is>
-      </c>
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Anatomie</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Catalogue espèces et parties compatibles</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/carcass-anatomy-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Stock explicite ; synthétique sans chair et xéno sans peau universelle.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="36" customHeight="1">
-      <c r="A23" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-19</t>
-        </is>
-      </c>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C23" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Anatomie</t>
-        </is>
-      </c>
-      <c r="D23" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Dommages mêlée/tir/surkill et analyse</t>
-        </is>
-      </c>
-      <c r="E23" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/carcass-anatomy-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F23" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Qualité reproductible annoncée, pas de nouveau tirage sur reload.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="36" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-20</t>
-        </is>
-      </c>
-      <c r="B24" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Anatomie</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Interruption/dépôt plein avant dernier tick</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/hunt-carcass-runtime-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Aucune partie consommée ni prise inventée.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="36" customHeight="1">
-      <c r="A25" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-21</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C25" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Anatomie</t>
-        </is>
-      </c>
-      <c r="D25" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Prélèvement puis succès/échec</t>
-        </is>
-      </c>
-      <c r="E25" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/hunt-carcass-runtime-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F25" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Succès verse identité/qualité exacte ; échec n'accorde pas le stock.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="36" customHeight="1">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-22</t>
-        </is>
-      </c>
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Charge</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Budgets scout24/18, hunter36/24, berserker52/30</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/harvest-inventory-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Masses/volumes calculés depuis les pièces ; refus atomique si dépassement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="36" customHeight="1">
-      <c r="A27" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-23</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C27" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Charge</t>
-        </is>
-      </c>
-      <c r="D27" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Plein déplacement/saut/grimpe/bruit</t>
-        </is>
-      </c>
-      <c r="E27" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/harvest-inventory-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F27" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Coefficients bornés .68/.84/1.6/1.8 aux limites.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="36" customHeight="1">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-24</t>
-        </is>
-      </c>
-      <c r="B28" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Charge</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Dépôt/reprise et campagne répétée</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/harvest-inventory-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Aucune perte silencieuse ni duplication des IDs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="36" customHeight="1">
-      <c r="A29" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-25</t>
-        </is>
-      </c>
-      <c r="B29" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C29" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Entretien</t>
-        </is>
-      </c>
-      <c r="D29" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Succès vs interruption/rejeu</t>
-        </is>
-      </c>
-      <c r="E29" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/harvest-inventory-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F29" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5 points par opération achevée, reçu unique, condition0..100.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="36" customHeight="1">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-26</t>
-        </is>
-      </c>
-      <c r="B30" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Entretien</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Réparation outil0 et aucune marque</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/harvest-inventory-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Affûtage gratuit et campagne débloquable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="36" customHeight="1">
-      <c r="A31" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-27</t>
-        </is>
-      </c>
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C31" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Atelier</t>
-        </is>
-      </c>
-      <c r="D31" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4 phasescoûts2/4/3/5 gestes3/4/5/3</t>
-        </is>
-      </c>
-      <c r="E31" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/harvest-inventory-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F31" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Transitions ordonnées, aucun progrès en absence, qualité conservée.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="36" customHeight="1">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-28</t>
-        </is>
-      </c>
-      <c r="B32" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Atelier</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Double clic et erreur durabilité</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/conservation-persistence-ui-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Coût/statut confirmés ensemble ; aucune réussite prématurée.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="36" customHeight="1">
-      <c r="A33" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-29</t>
-        </is>
-      </c>
-      <c r="B33" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C33" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Atelier</t>
-        </is>
-      </c>
-      <c r="D33" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Archive explicite pièce montée</t>
-        </is>
-      </c>
-      <c r="E33" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/harvest-inventory-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F33" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Réserve compte possession/qualité et libère le dépôt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="36" customHeight="1">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-30</t>
-        </is>
-      </c>
-      <c r="B34" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Accessibilité</t>
-        </is>
-      </c>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fenêtres normal/generous/unlimited</t>
-        </is>
-      </c>
-      <c r="E34" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/hunt-accessibility-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Règle réelle exécutée ; aucune prise automatique ni malus caché.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="36" customHeight="1">
-      <c r="A35" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-31</t>
-        </is>
-      </c>
-      <c r="B35" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C35" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Accessibilité</t>
-        </is>
-      </c>
-      <c r="D35" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Confirmpress/hold/toggle et annulation</t>
-        </is>
-      </c>
-      <c r="E35" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/hunt-accessibility-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F35" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Un acte par glyph, maintien min.35 s, bascule réarmée par nouveau glyph.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="36" customHeight="1">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-32</t>
-        </is>
-      </c>
-      <c r="B36" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C36" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Accessibilité</t>
-        </is>
-      </c>
-      <c r="D36" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Remapmanette +focus perdu</t>
-        </is>
-      </c>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/hunt-accessibility-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Permutation sans commande perdue ; bascule désarmée au blur.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="36" customHeight="1">
-      <c r="A37" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-33</t>
-        </is>
-      </c>
-      <c r="B37" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C37" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Accessibilité</t>
-        </is>
-      </c>
-      <c r="D37" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Migration et sérialisation réglages</t>
-        </is>
-      </c>
-      <c r="E37" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/hunt-accessibility-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F37" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Valeurs futures/malformed normalisées, latches transitoires non persistés.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="36" customHeight="1">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-34</t>
-        </is>
-      </c>
-      <c r="B38" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C38" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Écosystème</t>
-        </is>
-      </c>
-      <c r="D38" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Témoin visible vs derrière mur</t>
-        </is>
-      </c>
-      <c r="E38" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/corpse-discovery-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F38" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vision réelle déclenche un événement local unique.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="36" customHeight="1">
-      <c r="A39" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-35</t>
-        </is>
-      </c>
-      <c r="B39" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C39" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Écosystème</t>
-        </is>
-      </c>
-      <c r="D39" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Radio bornée, investigation et animaux</t>
-        </is>
-      </c>
-      <c r="E39" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/corpse-discovery-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F39" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Profils distincts, pas de boucle oualerte globale.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="36" customHeight="1">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-36</t>
-        </is>
-      </c>
-      <c r="B40" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Écosystème</t>
-        </is>
-      </c>
-      <c r="D40" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Budget et checkpoint</t>
-        </is>
-      </c>
-      <c r="E40" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/corpse-discovery-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F40" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">File/traitement bornés et identités restaurées sans rejouer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="42" customHeight="1">
-      <c r="A41" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-37</t>
-        </is>
-      </c>
-      <c r="B41" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C41" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Navigateur</t>
-        </is>
-      </c>
-      <c r="D41" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Paramètres natifs et téléphone390 px</t>
-        </is>
-      </c>
-      <c r="E41" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">scripts/qa-hunt-mechanics-browser-v112.mjs</t>
-        </is>
-      </c>
-      <c r="F41" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vrais composants utilisables ; stockage natif de fixture ; captures inspectables.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="36" customHeight="1">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-38</t>
-        </is>
-      </c>
-      <c r="B42" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Navigateur</t>
-        </is>
-      </c>
-      <c r="D42" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Atelier manuel jusqu'au montage puisréserve</t>
-        </is>
-      </c>
-      <c r="E42" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">scripts/qa-hunt-mechanics-browser-v112.mjs</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vrai panneau et règles, aucune écriture avant acknowledgement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="36" customHeight="1">
-      <c r="A43" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-39</t>
-        </is>
-      </c>
-      <c r="B43" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C43" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Navigateur</t>
-        </is>
-      </c>
-      <c r="D43" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Rites natifs flayinterrompu et terminé</t>
-        </is>
-      </c>
-      <c r="E43" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">scripts/qa-hunt-mechanics-browser-v112.mjs</t>
-        </is>
-      </c>
-      <c r="F43" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vraie mort, vrai handler AST et simulation ; un corps.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="36" customHeight="1">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-40</t>
-        </is>
-      </c>
-      <c r="B44" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C44" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Navigateur</t>
-        </is>
-      </c>
-      <c r="D44" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pendule clavier, tactile, manette émulée</t>
-        </is>
-      </c>
-      <c r="E44" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">scripts/qa-hunt-mechanics-browser-v112.mjs</t>
-        </is>
-      </c>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vrai polling/matchinginput/mouvement/rendu de repli ; vitesse réelle.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="36" customHeight="1">
-      <c r="A45" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA112-41</t>
-        </is>
-      </c>
-      <c r="B45" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
       <c r="C45" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Excel</t>
@@ -7669,19 +7669,19 @@
       </c>
       <c r="F45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Octets identiques au JSON ; ZIP/XML indépendant valide.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="42" customHeight="1">
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande node scripts/build-hunt-mechanics-workbook-v112.mjs --check ; python3 scripts/verify-hunt-mechanics-workbook-v112.py ; version avant consignation validée (427476 octets,2264 cellules,327 liens). La comparaison indépendante des nouveaux octets documentaires attend la CI de ce lot ; son résultat définitif figurera dans la PR. Aucun Excel natif.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="102" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">QA112-42</t>
         </is>
       </c>
-      <c r="B46" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
@@ -7701,19 +7701,19 @@
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freeze1386 vérifié, testsoriginaux et workbookinchangé ; aucune redirection prod.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="36" customHeight="1">
+          <t xml:space="preserve">commit ab47a9c2d2bf4b0a866c109efa2c96f68d526de8 ; commande node scripts/check-excel-history-v112.mjs --check --tests ; Copie privée depuis Git V110 épinglé : 1 386 entrées et préimages exactes des huit tests originaux vérifiées, 56 assertions et ancien XLSX inchangés ; aucune redirection du runtime V112. Résultat réel : 56 assertions originales PASS, SHA256 XLSX 0b7d7890c8d235a9cda0f6d61c62001efe150f2c4022924c20d88196afcdbd7c.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="117" customHeight="1">
       <c r="A47" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">QA112-43</t>
         </is>
       </c>
-      <c r="B47" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
@@ -7733,19 +7733,19 @@
       </c>
       <c r="F47" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freeze1433 vérifié, testsoriginaux et workbookinchangé.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="36" customHeight="1">
+          <t xml:space="preserve">commit ab47a9c2d2bf4b0a866c109efa2c96f68d526de8 ; commande node scripts/check-homeworld-history-v112.mjs --check --tests ; Copie privée depuis a5a951e : 1 433 entrées gelées et onze fichiers de tests originaux vérifiés, XLSX historique inchangé. Le test de publication gelée est ici ; les autres régressions V111 exécutent le runtime actuel. Résultat réel : 68 assertions originales PASS, SHA256 XLSX fa5ebf78a08c36b4a567246dfae41de535a8e36c7294ba33190e3e1e2ec9ad05.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="102" customHeight="1">
       <c r="A48" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">QA112-44</t>
         </is>
       </c>
-      <c r="B48" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
@@ -7755,7 +7755,7 @@
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TypeScript, lint, compilation et HTTP</t>
+          <t xml:space="preserve">TypeScript, lint, Next compilé, HTTP et régressions</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
@@ -7765,7 +7765,7 @@
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tous workflows finalHEAD verts, captures/limites consignées.</t>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; commande npm run typecheck ; node node_modules/next/dist/bin/next build --webpack ; npm run qa:next-production ; commande ESLint exacte dans .github/workflows/audit-v94.yml ; Résultats du run qualifié et commandes détaillés dans docs/qa/v112-hunt ; aucune performance sur appareil cible ni qualification de production déduite de cette CI.</t>
         </is>
       </c>
     </row>
@@ -7898,7 +7898,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
         </is>
       </c>
       <c r="C5" s="0" t="inlineStr">
@@ -7908,7 +7908,7 @@
       </c>
       <c r="D5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pendule avec longueur de corde, angle, vitesse tangentielle, tension et collision ; commande de pompage, lâcher libre et trajectoire lisible. Réserve d'endurance annoncée avant l'engagement.</t>
+          <t xml:space="preserve">Pendule natif : longueur, angle et vitesse tangentielle, pompage, friction, collision, endurance et lâcher sans boost.</t>
         </is>
       </c>
       <c r="E5" s="0" t="inlineStr">
@@ -7918,7 +7918,7 @@
       </c>
       <c r="F5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prototype jouable sur plusieurs longueurs ; pas d'énergie infinie, de traversée de murs ou de saut téléporté. Scénarios de relâchement, support perdu, pause et reprise.</t>
+          <t xml:space="preserve">Tests purs et HuntCanvas natif : plafonds, perte de support, checkpoint, épuisement et lâcher vers une autre liane. Pas de contrôleur physique qualifié.</t>
         </is>
       </c>
     </row>
@@ -7930,7 +7930,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -7940,7 +7940,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Composer des séquences de branches, troncs, lianes, corniches et points de repos. Définir les distances depuis les trajectoires réellement atteignables, avec route de repli et dangers lisibles.</t>
+          <t xml:space="preserve">Routes optionnelles dans le monde final : jusqu'à trois séquences selon géométrie, chacune de six vrais repos et accès depuis/vers le sol.</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -7950,11 +7950,11 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Parcours complets sur clavier, manette et tactile ; aucun passage obligatoire inaccessible à une armure autorisée.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="57" customHeight="1">
+          <t xml:space="preserve">72 traversées isolées natives (8 missions×3 armures×3 entrées normalisées) avec tous les contacts ; ennemis retirés pour isoler la locomotion. Aucun combat complet prétendu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="42" customHeight="1">
       <c r="A7" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">FUT-03</t>
@@ -7962,7 +7962,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
@@ -7972,7 +7972,7 @@
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Supports authorés avec hauteur, solidité, capacité de masse et espace libre. Transport et attache séparés ; interruption sûre et corps unique. Rendu et témoins placés au nouvel ancrage.</t>
+          <t xml:space="preserve">Préparer, porter puis suspendre le même acteur mort ; sockets arbre/chaîne avec dimensions, masse, volume libre, distance et visibilité réelles.</t>
         </is>
       </c>
       <c r="E7" s="0" t="inlineStr">
@@ -7982,7 +7982,7 @@
       </c>
       <c r="F7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tests de masse, support disparu, occlusion et sauvegarde ; aucune suspension acceptée depuis une décoration ou un support inventé.</t>
+          <t xml:space="preserve">Tests natifs : murs, transport bloqué, support perdu, source retirée au restore ; aucune décoration inventée comme ancrage.</t>
         </is>
       </c>
     </row>
@@ -7994,7 +7994,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -8004,7 +8004,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Définir par espèce les parties disponibles et leurs dépendances : peau, crâne, mandibule, colonne ou autre organe. Stock fini par corps ; compatibilité entre gestes et qualité.</t>
+          <t xml:space="preserve">Catalogue explicite de 39 espèces : peau, tissus et os secondaires uniquement lorsque disponibles ; stocks finis, gestes distincts, pièces identifiées.</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Catalogue sourcé, rendu disponible, inventaire limité et absence de duplication après interruption/reprise. Aucune partie universelle sur toutes les espèces.</t>
+          <t xml:space="preserve">Prérequis, interruption, capacité pleine, extraction et identité/qualité vérifiés automatiquement. Les trophées principaux historiques gardent leur règle distincte.</t>
         </is>
       </c>
     </row>
@@ -8026,7 +8026,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
@@ -8036,7 +8036,7 @@
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Séparer état initial de la proie, dommages causés aux parties et précision du prélèvement. Montrer le risque et la valeur potentielle avant de confirmer un geste irréversible.</t>
+          <t xml:space="preserve">Intégrité déterministe liée aux dégâts mêlée/tir/surkill ; analyse réduit la pénalité d'inconnu et aperçu par partie avant confirmation.</t>
         </is>
       </c>
       <c r="E9" s="0" t="inlineStr">
@@ -8046,7 +8046,7 @@
       </c>
       <c r="F9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Critères compréhensibles et reproductibles ; aucun malus invisible ou simple hasard impossible à lire.</t>
+          <t xml:space="preserve">Tests purs/natifs des coefficients et des dommages cumulés, qualité bornée et réutilisation du même état à la reprise ; pas d'étude de compréhension humaine.</t>
         </is>
       </c>
     </row>
@@ -8058,7 +8058,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -8068,7 +8068,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Masse et volume par prise, méthode de portage, limites d'armure et influence explicite sur saut, escalade et bruit. Dépôt temporaire ou rappel d'extraction avec coût annoncé.</t>
+          <t xml:space="preserve">Masse/volume des nouvelles pièces anatomiques et du corps porté ; limites par armure et effets explicites sur mouvement, saut, grimpe, bruit.</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -8078,11 +8078,11 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Règles communes inventaire/locomotion ; refus clair du surpoids et politique sans perte silencieuse lorsque l'emport est plein.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="57" customHeight="1">
+          <t xml:space="preserve">Sac de pause avec dépôt/reprise physique, collision/LOS et registre unique ; seuls portés exportés. Les anciens TrophyClaim ne reçoivent pas de poids supplémentaire.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="42" customHeight="1">
       <c r="A11" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">FUT-07</t>
@@ -8090,7 +8090,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
@@ -8100,7 +8100,7 @@
       </c>
       <c r="D11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Introduire précision, usure et entretien seulement si le joueur dispose d'un moyen clair de prévoir puis réparer. Séparer coût au démarrage, interruption et coût au succès.</t>
+          <t xml:space="preserve">Outil borné 0..100 ; 5 points par dépeçage/prélèvement achevé, durée jusqu'à×1,65 ; prévision réelle avant geste et affûtage gratuit.</t>
         </is>
       </c>
       <c r="E11" s="0" t="inlineStr">
@@ -8110,7 +8110,7 @@
       </c>
       <c r="F11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aucun double coût après reprise ; aucun blocage définitif de campagne si l'outil est abîmé. Économie testée avant fixation de chiffres.</t>
+          <t xml:space="preserve">Tests natifs de durée, reçus et interruption ; réparation à zéro marque vérifiée. L'usure acquise subsiste même si la mission échoue ensuite.</t>
         </is>
       </c>
     </row>
@@ -8122,7 +8122,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -8132,7 +8132,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nettoyage, traitement, séchage et montage avec files de travaux et états persistants. Le trophée possédé reste distinct de son entrée de collection ou de son exposition.</t>
+          <t xml:space="preserve">Nettoyer, traiter, sécher et monter par gestes manuels persistants ; coûts 2/4/3/5, unités 3/4/5/3, réserve explicite comptée.</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -8142,7 +8142,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Opérations idempotentes et coût lisible ; sauvegarde confirmée avant succès affiché ; aucun achèvement du temps réel sans règle explicite.</t>
+          <t xml:space="preserve">Réducteurs, acknowledgements et panneau React testés. Avance du calendrier simulée jusqu'en 2036 n'avance aucun travail ; aucune maturation réelle hors jeu.</t>
         </is>
       </c>
     </row>
@@ -8154,7 +8154,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
         </is>
       </c>
       <c r="C13" s="0" t="inlineStr">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Options de maintien/bascule, fenêtres ajustables, glyphes lisibles, alternatives au seul code couleur et commandes remappables. Indiquer les effets éventuels sur score avant le choix.</t>
+          <t xml:space="preserve">Fenêtres normale/large/sans limite, confirmation pression/maintien/bascule, glyphes lisibles, visée/prise basculées et douze commandes manette remappables.</t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr">
@@ -8174,11 +8174,11 @@
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Essais sur petits écrans et différentes entrées ; toutes les actions restent réalisables sans précision temporelle non expliquée.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="57" customHeight="1">
+          <t xml:space="preserve">Natif et Chromium : profils persistés, compteurs, remap, viewport390, menu corporel manette par défaut/remappée. Aucun appareil physique ni score d'une chasse complète qualifié.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="42" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">FUT-10</t>
@@ -8186,7 +8186,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -8196,7 +8196,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Différencier témoin qui voit un corps, alerte radio, investigation d'allié et peur d'une zone ; conserver l'identité des événements. Les bêtes ont des comportements propres au lieu d'une peur humaine.</t>
+          <t xml:space="preserve">Découverte locale par vue, odeur ou radio à un saut ; identités conservées, réactions animales distinctes et files bornées.</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -8206,7 +8206,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Budget IA mesuré, propagation bornée et sauvegarde cohérente ; pas d'alerte mondiale déclenchée par une trace invisible.</t>
+          <t xml:space="preserve">Tests des murs, visibilité, destinataires, rôles et reprise. Les plafonds de traitement sont vérifiés, sans mesure de performance matérielle.</t>
         </is>
       </c>
     </row>
@@ -8216,9 +8216,9 @@
           <t xml:space="preserve">FUT-11</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NON_QUALIFIE</t>
         </is>
       </c>
       <c r="C15" s="0" t="inlineStr">
@@ -8228,7 +8228,7 @@
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tutoriel court sur prise, bond, récupération et choix de route ; afficher l'action disponible et l'état d'outil près du corps sans encombrer le combat.</t>
+          <t xml:space="preserve">Guide contextuel implémenté, commandes réelles, épuisement, corps/trophée/extraction et choix de route distingués ; états React testés.</t>
         </is>
       </c>
       <c r="E15" s="0" t="inlineStr">
@@ -8238,7 +8238,7 @@
       </c>
       <c r="F15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Un nouveau joueur distingue corps, trophée et objectif d'extraction ; sorties et annulations compréhensibles.</t>
+          <t xml:space="preserve">NON_QUALIFIE pour compréhension d'un nouveau joueur et sorties comprises sans aide humaine ; seuls le rendu, le texte et les chemins logiciels sont vérifiés.</t>
         </is>
       </c>
     </row>
@@ -8248,9 +8248,9 @@
           <t xml:space="preserve">FUT-12</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">IMPLEMENTE_A_VALIDER</t>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NON_QUALIFIE</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -8260,7 +8260,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Relier les mécaniques à des chasses complètes, à toutes les armures admissibles et aux contraintes de performance. Conserver les limites entre test unitaire, navigateur et partie jouée.</t>
+          <t xml:space="preserve">Qualification automatique implémentée : matrice native 72 traversées, registres/transactions, 18 groupes Chromium et captures inspectées ; CI et historique séparés.</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
@@ -8270,7 +8270,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Parcours répétés sur appareils cibles, captures inspectées, absence d'erreurs et résultats documentés avec commit et périmètre exacts.</t>
+          <t xml:space="preserve">NON_QUALIFIE pour campagne interactive de combat complète, novice, téléphone/manette physiques et performance sur matériel cible. Les résultats automatisés bornés restent détaillés dans Qualification/Preuves.</t>
         </is>
       </c>
     </row>
@@ -8363,113 +8363,113 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="42" customHeight="1">
+    <row r="5" ht="72" customHeight="1">
       <c r="A5" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">PRF112-01</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tests natifs</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">237/237 tests V112, dont 72 traversées et quatre cas longs supports/plafond.</t>
+        </is>
+      </c>
+      <c r="E5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://github.com/darknigthmare/yautja-la-longue-chasse/actions/runs/40673101025</t>
+        </is>
+      </c>
+      <c r="F5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit e407979502d1cd4986e2e1810a4ed013f8abac8a ; merge exécuté37c472f2f727ae56cea52708a4c1e4922348fe82, arbre identique e1b5e0cec9da90e2efaeb879630545b1e6b862e0 ; commande node --experimental-strip-types --test --test-reporter=spec --test-concurrency=1 tests/*-v112.test.mjs ; PASS0fail0skip.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="87" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PRF112-02</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Navigateur</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">18 groupes Chromium PASS,0 exception pageerror ; cinq PNG conservés et inspectés.</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://github.com/darknigthmare/yautja-la-longue-chasse/actions/runs/40667918140</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">commit ab47a9c2d2bf4b0a866c109efa2c96f68d526de8 ; merge exécuté87a66e187a94616e46c657876d93aaaa933ba868, arbre identique ; commande node scripts/qa-hunt-mechanics-browser-v112.mjs. PNG/rapport dans docs/qa/v112-hunt au commit documentaire, pas au SHA antérieur. Ces captures ne prétendent pas qualifier les longues lianes du correctif suivant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="72" customHeight="1">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PRF112-03</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">A_EXECUTER</t>
         </is>
       </c>
-      <c r="C5" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tests natifs</t>
-        </is>
-      </c>
-      <c r="D5" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">node --experimental-strip-types --test --test-concurrency=1 tests/*-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="E5" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tests/hunt-canopy-runtime-v112.test.mjs</t>
-        </is>
-      </c>
-      <c r="F5" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Résultat à consigner depuis GitHub Actions sur le commit intégré.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PRF112-02</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Excel déterministe</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Contrôle binaire du classeur documentaire livré.</t>
+        </is>
+      </c>
+      <c r="E7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/build-hunt-mechanics-workbook-v112.mjs</t>
+        </is>
+      </c>
+      <c r="F7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Générateur et version avant consignation PASS au commit e407979502d1cd4986e2e1810a4ed013f8abac8a (427476 octets). Nouveaux octets avec preuves à comparer par la CI de ce lot ; résultat définitif dans la PR, sans inventer un SHA documentaire futur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="57" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PRF112-04</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">A_EXECUTER</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Navigateur</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">node scripts/qa-hunt-mechanics-browser-v112.mjs</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">scripts/qa-hunt-mechanics-browser-v112.mjs</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Rapport et captures dans outputs/qa-hunt-v112 ; pas de qualification matériel physique.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PRF112-03</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
-      <c r="C7" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Excel déterministe</t>
-        </is>
-      </c>
-      <c r="D7" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">node scripts/build-hunt-mechanics-workbook-v112.mjs --check</t>
-        </is>
-      </c>
-      <c r="E7" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">scripts/build-hunt-mechanics-workbook-v112.mjs</t>
-        </is>
-      </c>
-      <c r="F7" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Comparaison binaire ; ne lance pas Excel.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PRF112-04</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
-        </is>
-      </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Excel indépendant</t>
@@ -8477,7 +8477,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">python3 scripts/verify-hunt-mechanics-workbook-v112.py</t>
+          <t xml:space="preserve">Contrôle indépendant ZIP/XML du classeur documentaire livré.</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -8487,19 +8487,19 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ZIP, CRC, XML, cellules, liens, noms et filtres.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="36" customHeight="1">
+          <t xml:space="preserve">Avant consignation :2 264 cellules/327 liens PASS au commit e407979502d1cd4986e2e1810a4ed013f8abac8a. Vérification des contenus documentaires mis à jour attend la CI de ce lot ; aucun moteur Excel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="87" customHeight="1">
       <c r="A9" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">PRF112-05</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
@@ -8514,24 +8514,24 @@
       </c>
       <c r="E9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/check-excel-history-v112.mjs</t>
+          <t xml:space="preserve">https://github.com/darknigthmare/yautja-la-longue-chasse/actions/runs/40667918140</t>
         </is>
       </c>
       <c r="F9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Régressions actuelles restent distinctes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="36" customHeight="1">
+          <t xml:space="preserve">commit ab47a9c2d2bf4b0a866c109efa2c96f68d526de8 ; commande node scripts/check-excel-history-v112.mjs --check --tests ; contexte dff1f6734284891b5a24238f890070616a8325cc,1 386 empreintes,8 fichiers / 56 assertions originales PASS ; XLSX de 6 260 095 octets inchangé. Aucun test du runtime courant déduit de ce rejeu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="87" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">PRF112-06</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A_EXECUTER</t>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_AUTOMATISE</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -8546,12 +8546,12 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/check-homeworld-history-v112.mjs</t>
+          <t xml:space="preserve">https://github.com/darknigthmare/yautja-la-longue-chasse/actions/runs/40667918140</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Code à son commit a5 a951 e3 f6 dbb3 fa399 bd38 f774 a1 f0 b6 ec58 f5 e.</t>
+          <t xml:space="preserve">commit ab47a9c2d2bf4b0a866c109efa2c96f68d526de8 ; commande node scripts/check-homeworld-history-v112.mjs --check --tests ; contexte a5a951e3f6dbb3fa399bd38f774a1f0b6ec58f5e,1 433 empreintes,11 fichiers / 68 assertions originales PASS ; XLSX de 8 150 642 octets inchangé. Séparément119régressions V111 actuelles PASS.</t>
         </is>
       </c>
     </row>
@@ -10548,7 +10548,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="36" customHeight="1">
+    <row r="9" ht="42" customHeight="1">
       <c r="A9" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">CAN112-05</t>
@@ -10566,7 +10566,7 @@
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Haut/Bas ajustent la longueur à80 px/s entre70 px et hauteur du support.</t>
+          <t xml:space="preserve">Haut/Bas ajustent la longueur à80 px/s entre70 px et min(hauteur du support,2048 px).</t>
         </is>
       </c>
       <c r="E9" s="0" t="inlineStr">
@@ -10576,7 +10576,7 @@
       </c>
       <c r="F9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pas de corde négative ni extension hors support.</t>
+          <t xml:space="preserve">Longues lianes Oseris862/1054 px admises ; saisie dépassant le plafond ou état non fini refusés avant simulation.</t>
         </is>
       </c>
     </row>
@@ -11265,7 +11265,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="36" customHeight="1">
+    <row r="7" ht="42" customHeight="1">
       <c r="A7" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">SUS112-03</t>
@@ -11283,7 +11283,7 @@
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Corps transportable jusqu'à170 kg selon règle explicite.</t>
+          <t xml:space="preserve">Masse de gameplay = arrondi(borne(largeur×hauteur/60, 12, 300)) kg ; transport possible jusqu'à170 kg.</t>
         </is>
       </c>
       <c r="E7" s="0" t="inlineStr">
@@ -11293,7 +11293,7 @@
       </c>
       <c r="F7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Refus annoncé avant mutation.</t>
+          <t xml:space="preserve">Recalculée depuis l'acteur réel, y compris anciens checkpoints ; dimensions en pixels et valeurs non canoniques.</t>
         </is>
       </c>
     </row>
@@ -13616,7 +13616,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="36" customHeight="1">
+    <row r="5" ht="42" customHeight="1">
       <c r="A5" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">CHA112-01</t>
@@ -13634,7 +13634,7 @@
       </c>
       <c r="D5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Masse et volume calculés depuis les spécimens réellement présents.</t>
+          <t xml:space="preserve">Masse et volume des nouveaux prélèvements anatomiques portés, plus masse du corps porté, recomptés depuis le registre canonique.</t>
         </is>
       </c>
       <c r="E5" s="0" t="inlineStr">
@@ -13644,7 +13644,7 @@
       </c>
       <c r="F5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Un total sauvegardé seul n'accorde pas de capacité.</t>
+          <t xml:space="preserve">Les TrophyClaim principaux/secondaires historiques conservent leur contrat de collection et n'ajoutent pas de poids dans ce lot.</t>
         </is>
       </c>
     </row>
@@ -13840,7 +13840,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="36" customHeight="1">
+    <row r="12" ht="57" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">CHA112-08</t>
@@ -13858,17 +13858,17 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dépôt temporaire et reprise gardent chaque identité.</t>
+          <t xml:space="preserve">Dans le sac de pause, déposer/reprendre les nouvelles parties anatomiques au sol conserve leur identité canonique unique.</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">app/game/systems/harvestInventoryV112.ts</t>
+          <t xml:space="preserve">app/game/systems/fieldStashV112.ts</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Refus de reprise plein sans perte silencieuse.</t>
+          <t xml:space="preserve">Reprise à110 px, visibilité/appui/capacité ; gravité1850 px/s², chute plafonnée1200 px/s et collision balayée. Registre canonique borné64 ; seuls objets portés exportés.</t>
         </is>
       </c>
     </row>

</xml_diff>